<commit_message>
Reemplazar el Excel de control por JSON editable desde el panel
- config/control_plataforma.json sustituye a control_plataforma.xlsx
  como fuente única (mismo contenido: 64 parámetros, 21 APIs, 4 cuentas
  de servicio, 30 permisos, 12 usuarios, 4 datasets, 30 tablas, 240
  columnas, 2 secretos); build_config() no cambió, solo la lectura
- ops.py: read_excel() -> read_config() (lee el JSON en vez de abrir
  un .xlsx); ya no depende de openpyxl para la configuración
- panel/: pestañas por sección (Parámetros + tablas editables con
  agregar/quitar fila para usuarios, permisos, cuentas, APIs); las
  secciones que son contrato con SQL/Spark/Terraform (datasets,
  tablas, columnas, secretos) se muestran de solo lectura con aviso
- README, DEPLOY.md y la matriz de auditoría actualizados

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MgiFcvhexL3jkhqY5yJgLS
</commit_message>
<xml_diff>
--- a/docs/gestion/Matriz_Auditoria_Proyecto.xlsx
+++ b/docs/gestion/Matriz_Auditoria_Proyecto.xlsx
@@ -90,7 +90,7 @@
     <t xml:space="preserve">Estado se elige en la hoja Matriz (lista desplegable); '¿Hecho?', perfiles y resumen se recalculan solos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Despliegue: orden de comandos. Parámetros, nombres, tablas, columnas, usuarios y permisos: config/control_plataforma.xlsx.</t>
+    <t xml:space="preserve">Despliegue: orden de comandos. Parámetros, nombres, tablas, columnas, usuarios y permisos: config/control_plataforma.json (editable con `python ops.py panel`).</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -384,7 +384,7 @@
     <t xml:space="preserve">Terraform base</t>
   </si>
   <si>
-    <t xml:space="preserve">Buckets, BigQuery, Pub/Sub+DLQ, IAM, Artifact Registry, budget (valores desde el Excel de control)</t>
+    <t xml:space="preserve">Buckets, BigQuery, Pub/Sub+DLQ, IAM, Artifact Registry, budget (valores desde el JSON de control)</t>
   </si>
   <si>
     <t xml:space="preserve">infra/terraform/</t>
@@ -471,13 +471,13 @@
     <t xml:space="preserve">Git inicializado localmente</t>
   </si>
   <si>
-    <t xml:space="preserve">Excel de control de la plataforma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parámetros, APIs, cuentas, permisos, usuarios, datasets, tablas, columnas y secretos en un solo Excel validado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">config/control_plataforma.xlsx</t>
+    <t xml:space="preserve">JSON de control de la plataforma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parámetros, APIs, cuentas, permisos, usuarios, datasets, tablas, columnas y secretos en un solo JSON validado, editable con el panel web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">config/control_plataforma.json</t>
   </si>
   <si>
     <t xml:space="preserve">python ops.py config</t>
@@ -777,7 +777,7 @@
     <t xml:space="preserve">api/assistant.py</t>
   </si>
   <si>
-    <t xml:space="preserve">Excel: assistant_mode = gemini</t>
+    <t xml:space="preserve">config/control_plataforma.json: assistant_mode = gemini</t>
   </si>
   <si>
     <t xml:space="preserve">Reglas probadas con catálogo real; Gemini requiere GCP</t>
@@ -999,7 +999,7 @@
     <t xml:space="preserve">Acción</t>
   </si>
   <si>
-    <t xml:space="preserve">Insumo del Excel de control</t>
+    <t xml:space="preserve">Insumo del JSON de control</t>
   </si>
   <si>
     <t xml:space="preserve">Verificación</t>
@@ -1035,10 +1035,10 @@
     <t xml:space="preserve">D03</t>
   </si>
   <si>
-    <t xml:space="preserve">Completar el Excel de control</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Editar celdas amarillas de config/control_plataforma.xlsx (mínimo project_id y emails del equipo)</t>
+    <t xml:space="preserve">Completar el JSON de control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editar con `python ops.py panel` (o a mano) los campos marcados editables de config/control_plataforma.json: mínimo project_id y emails del equipo</t>
   </si>
   <si>
     <t xml:space="preserve">Parametros, Usuarios</t>
@@ -1209,7 +1209,7 @@
     <t xml:space="preserve">D16</t>
   </si>
   <si>
-    <t xml:space="preserve">Verificar contra el Excel</t>
+    <t xml:space="preserve">Verificar contra el JSON de control</t>
   </si>
   <si>
     <t xml:space="preserve">python ops.py verificar</t>
@@ -1254,7 +1254,7 @@
     <t xml:space="preserve">Costos reales</t>
   </si>
   <si>
-    <t xml:space="preserve">Consola: exportar facturación a BigQuery (dataset ops) -&gt; Excel billing_export_table -&gt; python ops.py costo-real</t>
+    <t xml:space="preserve">Consola: exportar facturación a BigQuery (dataset ops) -&gt; parámetro billing_export_table -&gt; python ops.py costo-real</t>
   </si>
   <si>
     <t xml:space="preserve">Parametros: billing_export_table</t>

</xml_diff>

<commit_message>
README con modelo de datos y reasignar D06/D19 a Estuardo Oliver
- README: sección "Fuente de datos" (H&M Kaggle, pública, sin
  redistribuir los CSV) y "Modelo de datos" con diagrama Mermaid del
  esquema estrella de Gold (dim_customer, dim_article, dim_date,
  dim_channel, fact_sales, fact_orders, reco_popular) y su origen
- Matriz de despliegue: D06 (Publicar repo) y D19 (Costos reales)
  reasignados de Winston Quispe a Estuardo Oliver

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MgiFcvhexL3jkhqY5yJgLS
</commit_message>
<xml_diff>
--- a/docs/gestion/Matriz_Auditoria_Proyecto.xlsx
+++ b/docs/gestion/Matriz_Auditoria_Proyecto.xlsx
@@ -4977,7 +4977,7 @@
         <v>349</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>350</v>
@@ -5276,7 +5276,7 @@
         <v>408</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>409</v>

</xml_diff>

<commit_message>
Actualizar matriz: proyecto GCP y repo GitHub ya hechos
- P1-17 (Crear proyecto GCP) y P1-18 (Publicar repositorio GitHub):
  Pendiente -> Hecho, con evidencia real (project tranquil-leaf-512618-b9
  con facturación, repo privado estuardoo/STYLUS con CI en verde)
- Paso 1 pasa de 71% a 81% (17/21 hechas, 1 pendiente: revisión y envío)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MgiFcvhexL3jkhqY5yJgLS
</commit_message>
<xml_diff>
--- a/docs/gestion/Matriz_Auditoria_Proyecto.xlsx
+++ b/docs/gestion/Matriz_Auditoria_Proyecto.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="416">
   <si>
     <t xml:space="preserve">Paso</t>
   </si>
@@ -450,70 +450,73 @@
     <t xml:space="preserve">ver hoja Despliegue D01-D04</t>
   </si>
   <si>
+    <t xml:space="preserve">Proyecto tranquil-leaf-512618-b9 con facturación vinculada; cuenta de servicio con rol owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publicar repositorio GitHub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crear repo privado, push y CI en verde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URL del repo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">git push -u origin main</t>
+  </si>
+  <si>
+    <t xml:space="preserve">github.com/estuardoo/STYLUS (privado); workflow ci en verde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JSON de control de la plataforma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parámetros, APIs, cuentas, permisos, usuarios, datasets, tablas, columnas y secretos en un solo JSON validado, editable con el panel web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">config/control_plataforma.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python ops.py config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 tablas, 240 columnas, 28 permisos, 6 usuarios app; CI verifica generados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orquestador de despliegue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un comando por paso, multiplataforma, con log matricial de tiempos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ops.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python ops.py todo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">config/estado/local probados; comandos de nube pendientes de GCP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión y envío Entrega 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión cruzada del Word y envío antes de 23:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Word enviado</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Publicar repositorio GitHub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crear repo privado, push y CI en verde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">URL del repo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">git push -u origin main</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Git inicializado localmente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JSON de control de la plataforma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parámetros, APIs, cuentas, permisos, usuarios, datasets, tablas, columnas y secretos en un solo JSON validado, editable con el panel web</t>
-  </si>
-  <si>
-    <t xml:space="preserve">config/control_plataforma.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python ops.py config</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 tablas, 240 columnas, 28 permisos, 6 usuarios app; CI verifica generados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orquestador de despliegue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un comando por paso, multiplataforma, con log matricial de tiempos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ops.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python ops.py todo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">config/estado/local probados; comandos de nube pendientes de GCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisión y envío Entrega 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisión cruzada del Word y envío antes de 23:59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Word enviado</t>
   </si>
   <si>
     <t xml:space="preserve">Desplegar infraestructura dev</t>
@@ -1884,7 +1887,7 @@
       </c>
       <c r="E2" s="2" t="n">
         <f aca="false">COUNTIFS(Matriz!$B$2:$B$52,$A2,Matriz!$N$2:$N$52,"Hecho")</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2" s="2" t="n">
         <f aca="false">COUNTIFS(Matriz!$B$2:$B$52,$A2,Matriz!$N$2:$N$52,"Listo para desplegar")</f>
@@ -1892,15 +1895,15 @@
       </c>
       <c r="G2" s="2" t="n">
         <f aca="false">COUNTIFS(Matriz!$B$2:$B$52,$A2,Matriz!$N$2:$N$52,"Pendiente")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2" s="3" t="n">
         <f aca="false">IF(D2&gt;0,E2/D2,0)</f>
-        <v>0.714285714285714</v>
+        <v>0.80952380952381</v>
       </c>
       <c r="I2" s="3" t="n">
         <f aca="false">IF(D2&gt;0,(E2+F2)/D2,0)</f>
-        <v>0.857142857142857</v>
+        <v>0.952380952380952</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1985,7 +1988,7 @@
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">SUM(E2:E4)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">SUM(F2:F4)</f>
@@ -1993,15 +1996,15 @@
       </c>
       <c r="G5" s="4" t="n">
         <f aca="false">SUM(G2:G4)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">IF(D5&gt;0,E5/D5,0)</f>
-        <v>0.352941176470588</v>
+        <v>0.392156862745098</v>
       </c>
       <c r="I5" s="5" t="n">
         <f aca="false">IF(D5&gt;0,(E5+F5)/D5,0)</f>
-        <v>0.705882352941177</v>
+        <v>0.745098039215686</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2891,7 +2894,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
         <v>135</v>
       </c>
@@ -2929,15 +2932,17 @@
       </c>
       <c r="M18" s="10"/>
       <c r="N18" s="10" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="O18" s="10" t="str">
         <f aca="false">IF(N18="Hecho","Sí","No")</f>
-        <v>No</v>
-      </c>
-      <c r="P18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>Sí</v>
+      </c>
+      <c r="P18" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>141</v>
       </c>
@@ -2979,11 +2984,11 @@
         <v>128</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>140</v>
+        <v>43</v>
       </c>
       <c r="O19" s="10" t="str">
         <f aca="false">IF(N19="Hecho","Sí","No")</f>
-        <v>No</v>
+        <v>Sí</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>146</v>
@@ -3131,7 +3136,7 @@
         <v>128</v>
       </c>
       <c r="N22" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O22" s="10" t="str">
         <f aca="false">IF(N22="Hecho","Sí","No")</f>
@@ -3156,16 +3161,16 @@
         <v>116</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J23" s="10" t="s">
         <v>135</v>
@@ -3179,7 +3184,7 @@
       </c>
       <c r="M23" s="10"/>
       <c r="N23" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O23" s="10" t="str">
         <f aca="false">IF(N23="Hecho","Sí","No")</f>
@@ -3189,7 +3194,7 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B24" s="11" t="n">
         <v>2</v>
@@ -3204,16 +3209,16 @@
         <v>37</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J24" s="10" t="s">
         <v>96</v>
@@ -3229,19 +3234,19 @@
         <v>50</v>
       </c>
       <c r="N24" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O24" s="10" t="str">
         <f aca="false">IF(N24="Hecho","Sí","No")</f>
         <v>No</v>
       </c>
       <c r="P24" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B25" s="11" t="n">
         <v>2</v>
@@ -3256,19 +3261,19 @@
         <v>37</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J25" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>41</v>
@@ -3288,12 +3293,12 @@
         <v>No</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B26" s="11" t="n">
         <v>2</v>
@@ -3308,19 +3313,19 @@
         <v>37</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J26" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K26" s="10" t="s">
         <v>41</v>
@@ -3341,7 +3346,7 @@
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B27" s="11" t="n">
         <v>2</v>
@@ -3353,22 +3358,22 @@
         <v>12</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J27" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>41</v>
@@ -3391,7 +3396,7 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B28" s="11" t="n">
         <v>2</v>
@@ -3403,19 +3408,19 @@
         <v>12</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J28" s="10" t="s">
         <v>96</v>
@@ -3436,12 +3441,12 @@
         <v>No</v>
       </c>
       <c r="P28" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B29" s="11" t="n">
         <v>2</v>
@@ -3453,16 +3458,16 @@
         <v>12</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="10" t="s">
@@ -3487,7 +3492,7 @@
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B30" s="11" t="n">
         <v>2</v>
@@ -3499,22 +3504,22 @@
         <v>12</v>
       </c>
       <c r="E30" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="J30" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="H30" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="J30" s="10" t="s">
-        <v>188</v>
       </c>
       <c r="K30" s="10" t="s">
         <v>50</v>
@@ -3534,12 +3539,12 @@
         <v>No</v>
       </c>
       <c r="P30" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B31" s="11" t="n">
         <v>2</v>
@@ -3551,22 +3556,22 @@
         <v>12</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J31" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K31" s="10" t="s">
         <v>42</v>
@@ -3589,7 +3594,7 @@
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B32" s="11" t="n">
         <v>2</v>
@@ -3601,19 +3606,19 @@
         <v>12</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J32" s="10"/>
       <c r="K32" s="10" t="s">
@@ -3632,12 +3637,12 @@
         <v>Sí</v>
       </c>
       <c r="P32" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B33" s="11" t="n">
         <v>2</v>
@@ -3652,13 +3657,13 @@
         <v>37</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I33" s="10"/>
       <c r="J33" s="10"/>
@@ -3681,7 +3686,7 @@
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B34" s="11" t="n">
         <v>2</v>
@@ -3696,19 +3701,19 @@
         <v>105</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J34" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K34" s="10" t="s">
         <v>69</v>
@@ -3731,7 +3736,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B35" s="11" t="n">
         <v>2</v>
@@ -3746,17 +3751,17 @@
         <v>105</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K35" s="10" t="s">
         <v>69</v>
@@ -3767,7 +3772,7 @@
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O35" s="10" t="str">
         <f aca="false">IF(N35="Hecho","Sí","No")</f>
@@ -3777,7 +3782,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B36" s="11" t="n">
         <v>2</v>
@@ -3792,17 +3797,17 @@
         <v>46</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K36" s="10" t="s">
         <v>42</v>
@@ -3815,7 +3820,7 @@
         <v>128</v>
       </c>
       <c r="N36" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O36" s="10" t="str">
         <f aca="false">IF(N36="Hecho","Sí","No")</f>
@@ -3825,7 +3830,7 @@
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B37" s="12" t="n">
         <v>3</v>
@@ -3837,19 +3842,19 @@
         <v>14</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I37" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J37" s="10"/>
       <c r="K37" s="10" t="s">
@@ -3870,12 +3875,12 @@
         <v>No</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B38" s="12" t="n">
         <v>3</v>
@@ -3887,19 +3892,19 @@
         <v>14</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J38" s="10"/>
       <c r="K38" s="10" t="s">
@@ -3918,12 +3923,12 @@
         <v>No</v>
       </c>
       <c r="P38" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B39" s="12" t="n">
         <v>3</v>
@@ -3935,19 +3940,19 @@
         <v>14</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J39" s="10" t="s">
         <v>96</v>
@@ -3970,12 +3975,12 @@
         <v>No</v>
       </c>
       <c r="P39" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B40" s="12" t="n">
         <v>3</v>
@@ -3987,16 +3992,16 @@
         <v>14</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
@@ -4019,7 +4024,7 @@
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B41" s="12" t="n">
         <v>3</v>
@@ -4031,19 +4036,19 @@
         <v>14</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J41" s="10"/>
       <c r="K41" s="10" t="s">
@@ -4067,7 +4072,7 @@
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B42" s="12" t="n">
         <v>3</v>
@@ -4082,16 +4087,16 @@
         <v>116</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J42" s="10" t="s">
         <v>96</v>
@@ -4112,12 +4117,12 @@
         <v>No</v>
       </c>
       <c r="P42" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B43" s="12" t="n">
         <v>3</v>
@@ -4132,16 +4137,16 @@
         <v>116</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J43" s="10" t="s">
         <v>141</v>
@@ -4165,7 +4170,7 @@
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B44" s="12" t="n">
         <v>3</v>
@@ -4180,19 +4185,19 @@
         <v>37</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J44" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K44" s="10" t="s">
         <v>41</v>
@@ -4205,19 +4210,19 @@
         <v>50</v>
       </c>
       <c r="N44" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O44" s="10" t="str">
         <f aca="false">IF(N44="Hecho","Sí","No")</f>
         <v>No</v>
       </c>
       <c r="P44" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B45" s="12" t="n">
         <v>3</v>
@@ -4232,17 +4237,17 @@
         <v>105</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K45" s="10" t="s">
         <v>69</v>
@@ -4255,7 +4260,7 @@
         <v>42</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O45" s="10" t="str">
         <f aca="false">IF(N45="Hecho","Sí","No")</f>
@@ -4265,7 +4270,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B46" s="12" t="n">
         <v>3</v>
@@ -4280,17 +4285,17 @@
         <v>105</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K46" s="10" t="s">
         <v>69</v>
@@ -4303,7 +4308,7 @@
         <v>50</v>
       </c>
       <c r="N46" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O46" s="10" t="str">
         <f aca="false">IF(N46="Hecho","Sí","No")</f>
@@ -4313,7 +4318,7 @@
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B47" s="12" t="n">
         <v>3</v>
@@ -4328,17 +4333,17 @@
         <v>100</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K47" s="10" t="s">
         <v>50</v>
@@ -4351,19 +4356,19 @@
         <v>41</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O47" s="10" t="str">
         <f aca="false">IF(N47="Hecho","Sí","No")</f>
         <v>No</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B48" s="12" t="n">
         <v>3</v>
@@ -4378,13 +4383,13 @@
         <v>85</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="10" t="s">
@@ -4401,7 +4406,7 @@
         <v>50</v>
       </c>
       <c r="N48" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O48" s="10" t="str">
         <f aca="false">IF(N48="Hecho","Sí","No")</f>
@@ -4411,7 +4416,7 @@
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B49" s="12" t="n">
         <v>3</v>
@@ -4426,13 +4431,13 @@
         <v>46</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
@@ -4457,7 +4462,7 @@
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B50" s="12" t="n">
         <v>3</v>
@@ -4472,17 +4477,17 @@
         <v>46</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="I50" s="10"/>
       <c r="J50" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K50" s="10" t="s">
         <v>69</v>
@@ -4495,7 +4500,7 @@
         <v>128</v>
       </c>
       <c r="N50" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O50" s="10" t="str">
         <f aca="false">IF(N50="Hecho","Sí","No")</f>
@@ -4505,7 +4510,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B51" s="12" t="n">
         <v>3</v>
@@ -4520,17 +4525,17 @@
         <v>46</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="K51" s="10" t="s">
         <v>42</v>
@@ -4543,7 +4548,7 @@
         <v>128</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O51" s="10" t="str">
         <f aca="false">IF(N51="Hecho","Sí","No")</f>
@@ -4553,7 +4558,7 @@
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B52" s="12" t="n">
         <v>3</v>
@@ -4568,19 +4573,19 @@
         <v>85</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J52" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K52" s="10" t="s">
         <v>50</v>
@@ -4591,7 +4596,7 @@
       </c>
       <c r="M52" s="10"/>
       <c r="N52" s="10" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="O52" s="10" t="str">
         <f aca="false">IF(N52="Hecho","Sí","No")</f>
@@ -4654,13 +4659,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>3</v>
@@ -4683,10 +4688,10 @@
         <v>42</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D2" s="2" t="n">
         <f aca="false">COUNTIF(Matriz!$K$2:$K$52,A2)</f>
@@ -4714,10 +4719,10 @@
         <v>50</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D3" s="2" t="n">
         <f aca="false">COUNTIF(Matriz!$K$2:$K$52,A3)</f>
@@ -4725,7 +4730,7 @@
       </c>
       <c r="E3" s="2" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$2:$K$52,$A3,Matriz!$N$2:$N$52,"Hecho")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F3" s="2" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$2:$K$52,$A3,Matriz!$N$2:$N$52,"Listo para desplegar")</f>
@@ -4733,11 +4738,11 @@
       </c>
       <c r="G3" s="2" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$2:$K$52,$A3,Matriz!$N$2:$N$52,"Pendiente")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H3" s="3" t="n">
         <f aca="false">IF(D3&gt;0,E3/D3,0)</f>
-        <v>0.277777777777778</v>
+        <v>0.388888888888889</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4745,10 +4750,10 @@
         <v>41</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D4" s="2" t="n">
         <f aca="false">COUNTIF(Matriz!$K$2:$K$52,A4)</f>
@@ -4776,10 +4781,10 @@
         <v>69</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D5" s="2" t="n">
         <f aca="false">COUNTIF(Matriz!$K$2:$K$52,A5)</f>
@@ -4836,10 +4841,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>28</v>
@@ -4848,10 +4853,10 @@
         <v>30</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4859,20 +4864,20 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F2" s="10"/>
       <c r="G2" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4880,22 +4885,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4903,22 +4908,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4926,20 +4931,20 @@
         <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F5" s="10"/>
       <c r="G5" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4947,20 +4952,20 @@
         <v>1</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F6" s="10"/>
       <c r="G6" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4968,22 +4973,22 @@
         <v>1</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>42</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4991,22 +4996,22 @@
         <v>2</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5014,10 +5019,10 @@
         <v>2</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>120</v>
@@ -5026,10 +5031,10 @@
         <v>50</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5037,22 +5042,22 @@
         <v>2</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5060,22 +5065,22 @@
         <v>2</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5083,22 +5088,22 @@
         <v>2</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5106,22 +5111,22 @@
         <v>2</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5129,22 +5134,22 @@
         <v>2</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5152,22 +5157,22 @@
         <v>2</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,22 +5180,22 @@
         <v>3</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5198,22 +5203,22 @@
         <v>3</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5221,22 +5226,22 @@
         <v>3</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5244,22 +5249,22 @@
         <v>3</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>69</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5267,22 +5272,22 @@
         <v>3</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>42</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5290,22 +5295,22 @@
         <v>3</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>